<commit_message>
Update defect analysis report and add root cause validation list (30 defects)
</commit_message>
<xml_diff>
--- a/backend/src/data/Customer Defects Created in Past 6 Months 2.xlsx
+++ b/backend/src/data/Customer Defects Created in Past 6 Months 2.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\AI Projects Update\AI Projects\CustomerDefectRootCauseAnalyzer\backend\src\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0DC3BAE4-AD34-4B18-AE38-C0424295B7DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B547E37-0C28-4470-9B19-8760D599F996}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16674,7 +16674,7 @@
   <dimension ref="A1:BE133"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="11.140625" style="6" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="28.28515625" style="6" customWidth="1"/>
     <col min="2" max="3" width="13.5703125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="34.42578125" customWidth="1"/>
     <col min="5" max="6" width="13.5703125" bestFit="1" customWidth="1"/>
@@ -16682,7 +16682,8 @@
     <col min="8" max="13" width="13.5703125" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="22" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="19.42578125" bestFit="1" customWidth="1"/>
-    <col min="16" max="25" width="13.5703125" bestFit="1" customWidth="1"/>
+    <col min="16" max="24" width="13.5703125" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="27" customWidth="1"/>
     <col min="26" max="26" width="13.5703125" style="11" bestFit="1" customWidth="1"/>
     <col min="27" max="53" width="13.5703125" bestFit="1" customWidth="1"/>
     <col min="54" max="54" width="13.5703125" style="13" bestFit="1" customWidth="1"/>

</xml_diff>